<commit_message>
test(report5): checkpoint planned API evidence and reconciled reports
</commit_message>
<xml_diff>
--- a/docs/report5/deliverables/Report5_Unit Test.xlsx
+++ b/docs/report5/deliverables/Report5_Unit Test.xlsx
@@ -2,103 +2,103 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R13851cc004a4404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F001" sheetId="2" r:id="R1910ae2d8a6b492b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F002" sheetId="3" r:id="R52635aefa9d54eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F003" sheetId="4" r:id="Re94bc5ea7b794ea2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F004" sheetId="5" r:id="R44d5b773d4b94a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F005" sheetId="6" r:id="R37a3f4c097464859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F006" sheetId="7" r:id="Rf841722f5f88468f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F007" sheetId="8" r:id="R0bf621ae7ef74043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F008" sheetId="9" r:id="R4e7e0d9aba2b4773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F009" sheetId="10" r:id="R2fea55039fc4430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F010" sheetId="11" r:id="Rcd4f777591054ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F011" sheetId="12" r:id="Rfcc8a75e07a14fef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F012" sheetId="13" r:id="R8a5370d9ac6d4e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F013" sheetId="14" r:id="Rfc96beea81a94fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F014" sheetId="15" r:id="R5e580a67d2884138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F015" sheetId="16" r:id="R099773fcad23473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F016" sheetId="17" r:id="R9daecff8b6a74ec8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F017" sheetId="18" r:id="R5586376881114aca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F018" sheetId="19" r:id="R4c3ccf84c59d4917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F019" sheetId="20" r:id="Rb54a7b739e2e4706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F020" sheetId="21" r:id="R5cd27c9aeba64e75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F021" sheetId="22" r:id="R77508b4fe4164180"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F022" sheetId="23" r:id="R59f4ecc785944921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F023" sheetId="24" r:id="R3d13254ec05e42c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F024" sheetId="25" r:id="R58b1d13027824ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F025" sheetId="26" r:id="R3fbe4d0bde7c4a03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F026" sheetId="27" r:id="Rc96eaf1ea44d46ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F027" sheetId="28" r:id="R4a63f0eef04a43ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F028" sheetId="29" r:id="R7b8d48a0cb8c4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F029" sheetId="30" r:id="Rb7ab4ec1aae24301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F030" sheetId="31" r:id="R307e02d18d1541c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F031" sheetId="32" r:id="R99963739f4a844e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F032" sheetId="33" r:id="R63c792d2cfde4f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F033" sheetId="34" r:id="Rc3735ade28904848"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F034" sheetId="35" r:id="R77024bc0375e4e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F035" sheetId="36" r:id="R9d8048f7d6714b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F036" sheetId="37" r:id="R67efef170c604ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F037" sheetId="38" r:id="R0a4dc4e1db1c40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F038" sheetId="39" r:id="Rb908cb4e424344c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F039" sheetId="40" r:id="R92105c18be064e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F040" sheetId="41" r:id="R7ebf949e5a694a27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F041" sheetId="42" r:id="R277a2dda1e714c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F042" sheetId="43" r:id="R51e08c2903a0469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F043" sheetId="44" r:id="R2cddd4e0c5c74292"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F044" sheetId="45" r:id="R7a180acc6c794f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F045" sheetId="46" r:id="Rb033df8ac8124e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F046" sheetId="47" r:id="R4b5d46882b9a4498"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F047" sheetId="48" r:id="R0bb7fec13f4f486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F048" sheetId="49" r:id="Rbcf9659b693243ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F049" sheetId="50" r:id="Rac686a8f61f74cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F050" sheetId="51" r:id="Re738499e51c44b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F051" sheetId="52" r:id="Rbd0351a440464658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F052" sheetId="53" r:id="R93a87bd714044c71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F053" sheetId="54" r:id="Re46fd5613b804590"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F054" sheetId="55" r:id="Rea5b33ad4cae4ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F055" sheetId="56" r:id="R2d1d1deb24fe4379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F056" sheetId="57" r:id="Re74c5c78c543444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F057" sheetId="58" r:id="R8987b6a7b33d4fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F058" sheetId="59" r:id="Rf9004193a5824c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F059" sheetId="60" r:id="R625c5a5fd5214e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F060" sheetId="61" r:id="R3d446140010a4e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F061" sheetId="62" r:id="Ra1695188e0574c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F062" sheetId="63" r:id="R62042c884abe4d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F063" sheetId="64" r:id="Refc8e7ac210e4f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F064" sheetId="65" r:id="R7a3ea23c1e474687"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F065" sheetId="66" r:id="R3c650c0b8b8a4d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F066" sheetId="67" r:id="R80725baf1aa14bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F067" sheetId="68" r:id="R2fe28acf33004107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F068" sheetId="69" r:id="R1eec1fa440504f5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F069" sheetId="70" r:id="Rdb5860017a5f4688"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F070" sheetId="71" r:id="R2f28abb339e2488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F071" sheetId="72" r:id="R58cf6d0dd84c43a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F072" sheetId="73" r:id="R93a48e9a8ceb4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F073" sheetId="74" r:id="R2aa4b13969a04640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F074" sheetId="75" r:id="Rc3118f8e07ee43ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F075" sheetId="76" r:id="Rc9a0526757c141b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F076" sheetId="77" r:id="R7b53364bbc304417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F077" sheetId="78" r:id="R90a3db99c61940ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F078" sheetId="79" r:id="Rcdb61cd8a3184330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F079" sheetId="80" r:id="R47be77b174274505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F080" sheetId="81" r:id="R7c87d7ab3b384d6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F081" sheetId="82" r:id="Rd6b262b9e85a4a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F082" sheetId="83" r:id="R9c38752ac4284eee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F083" sheetId="84" r:id="Rcc1139dfbab54fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F084" sheetId="85" r:id="R94fa4457553c4e5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F085" sheetId="86" r:id="Rb108e949b6ea4dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F086" sheetId="87" r:id="R85df016ac9254002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F087" sheetId="88" r:id="Rf5f6bd13813846e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F088" sheetId="89" r:id="R65b0903949fd4d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F089" sheetId="90" r:id="R1bdea86ed13d4e3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F090" sheetId="91" r:id="R34f9e057a20442c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F091" sheetId="92" r:id="Rf82bc3fdcd204ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F092" sheetId="93" r:id="Rd3d35b254e9d4cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F093" sheetId="94" r:id="R4bcb5a2b0d094aaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functions" sheetId="95" r:id="Rec1db2baadae461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="96" r:id="Ra9885d02096d4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guideline" sheetId="97" r:id="R89d7d4837f4a4028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R54064a8acc7740dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F001" sheetId="2" r:id="R7e3de14bd61f44bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F002" sheetId="3" r:id="Re2f3c8e4a07d4f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F003" sheetId="4" r:id="Rab4ee5e6744442cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F004" sheetId="5" r:id="Rec0a2a56aec24f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F005" sheetId="6" r:id="R9ff7cf52a8294128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F006" sheetId="7" r:id="R940283d5e97b49d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F007" sheetId="8" r:id="R29d8c6750ae44b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F008" sheetId="9" r:id="R2c2362b9265240ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F009" sheetId="10" r:id="Ra0efb20d89c94c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F010" sheetId="11" r:id="R4f4e30428df24c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F011" sheetId="12" r:id="Rb475828c1e574ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F012" sheetId="13" r:id="R18709b0cd6cc4e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F013" sheetId="14" r:id="R233e559629e0496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F014" sheetId="15" r:id="R5f736ef694e84efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F015" sheetId="16" r:id="R6764d79df68642d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F016" sheetId="17" r:id="R8dc440e4da3d4791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F017" sheetId="18" r:id="R64ad11f462a14049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F018" sheetId="19" r:id="R7b80b87b5be64470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F019" sheetId="20" r:id="Rf40e7dd8bdf04c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F020" sheetId="21" r:id="R229f625aceb04b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F021" sheetId="22" r:id="R6432aa7d54c54a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F022" sheetId="23" r:id="R7f83bed639fd4529"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F023" sheetId="24" r:id="R23e1320f0d174bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F024" sheetId="25" r:id="R362a9a103908427e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F025" sheetId="26" r:id="Rf05e7215251c4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F026" sheetId="27" r:id="R88cebe9ff3c44b94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F027" sheetId="28" r:id="R8d4ec29c6eb44857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F028" sheetId="29" r:id="Rd95e710ba636489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F029" sheetId="30" r:id="R2a3110adf7d8473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F030" sheetId="31" r:id="R7f8041324128406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F031" sheetId="32" r:id="R3340536ee52843fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F032" sheetId="33" r:id="Rab5b77f47aad46f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F033" sheetId="34" r:id="Ra62e8c47a819416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F034" sheetId="35" r:id="Rca77d723cfcb4615"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F035" sheetId="36" r:id="Re97a086795ae4800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F036" sheetId="37" r:id="R39acee8fe5614595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F037" sheetId="38" r:id="Ra1dbb27a67a74ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F038" sheetId="39" r:id="Rcbe6ff4caa72436d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F039" sheetId="40" r:id="R8a0687c0183a44ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F040" sheetId="41" r:id="Ra37002e125854712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F041" sheetId="42" r:id="Rcf810d188f0f489e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F042" sheetId="43" r:id="Rff884bdfcc384eb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F043" sheetId="44" r:id="Rb6335f98a00e4797"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F044" sheetId="45" r:id="R2a65f28a8f064c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F045" sheetId="46" r:id="Rae8b85f4115b4349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F046" sheetId="47" r:id="Rcb80648c672947ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F047" sheetId="48" r:id="R336c159a7a1443f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F048" sheetId="49" r:id="R4465e585a1a94821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F049" sheetId="50" r:id="R4d9f594308e44f8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F050" sheetId="51" r:id="Rb3c431ddbf054857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F051" sheetId="52" r:id="R3c56a52ef84e417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F052" sheetId="53" r:id="R8dfef552e13c431b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F053" sheetId="54" r:id="R426199d9cebb412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F054" sheetId="55" r:id="R159ae7c385984064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F055" sheetId="56" r:id="Rbf6a2b297fa94d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F056" sheetId="57" r:id="R5314ba10c2734f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F057" sheetId="58" r:id="R5dfff26ebbd0437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F058" sheetId="59" r:id="R9f4538bfbb97455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F059" sheetId="60" r:id="Rec3013d0abb54960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F060" sheetId="61" r:id="Rccb239776b9e4862"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F061" sheetId="62" r:id="R5ab1ed0837324ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F062" sheetId="63" r:id="R5493350ee86c4357"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F063" sheetId="64" r:id="R80e68f3d54674607"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F064" sheetId="65" r:id="R6d110b967b80427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F065" sheetId="66" r:id="Rae36f62a5f4c4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F066" sheetId="67" r:id="R06b2ef95994844ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F067" sheetId="68" r:id="Rb1c4463e7f0c4e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F068" sheetId="69" r:id="Ra0a8feee937449b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F069" sheetId="70" r:id="Ra473b222750c408c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F070" sheetId="71" r:id="Rfad7e66fdf874012"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F071" sheetId="72" r:id="Rf015370026044831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F072" sheetId="73" r:id="Re77a0d96bec14312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F073" sheetId="74" r:id="Rbb977bafa2424e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F074" sheetId="75" r:id="R1d0b3789d44f46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F075" sheetId="76" r:id="Rbd4af813d7eb4eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F076" sheetId="77" r:id="R5d9ea755f5ea4b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F077" sheetId="78" r:id="Rb12f8824edbe47ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F078" sheetId="79" r:id="R68e198ab97664b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F079" sheetId="80" r:id="R28d9cd4fb97141aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F080" sheetId="81" r:id="Rc6e7fa5463fa4543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F081" sheetId="82" r:id="R16c2d07efb4a447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F082" sheetId="83" r:id="Re3cbf81e3e764eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F083" sheetId="84" r:id="Re0086f7d94be4043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F084" sheetId="85" r:id="Rf2fd441e7b0a4562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F085" sheetId="86" r:id="Rcd0c52f3c4784498"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F086" sheetId="87" r:id="R26c018e715df4228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F087" sheetId="88" r:id="Ra72caef5b4884d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F088" sheetId="89" r:id="R7dc2a0f65f8f4b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F089" sheetId="90" r:id="R0992982d4d7540ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F090" sheetId="91" r:id="R147650b2409d491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F091" sheetId="92" r:id="R685ced85884b403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F092" sheetId="93" r:id="R2d6b5b9a45974089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F093" sheetId="94" r:id="R6e47c04da7784390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functions" sheetId="95" r:id="Rea0defa7ac264ec8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="96" r:id="R6f9d9a0f79e6483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guideline" sheetId="97" r:id="R4624b3091d0d4dc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34836,6 +34836,14 @@
         <x:v>R5-DEF-001 — Open / Fail: Approved registration accepts request-more-info. Evidence: integration.trx, Registration_ApprovedRequest_CannotBeReopenedForDocuments. This is an integration failure, not a failed unit case; the 203 unit results remain Passed.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13" ht="85" customHeight="1">
+      <x:c r="A13" s="9" t="str">
+        <x:v>Related authorization defect</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="str">
+        <x:v>R5-DEF-002 — Open / Fail: Reader can create a book via POST /api/v1/books/form (HTTP 201; persisted=True). Evidence: planned-api/planned-api.trx, ST_02_3_ReaderCannotMutateInventory. Integration defect; unit verdicts unchanged.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>